<commit_message>
Daily NSE scan: 2026-09-18
</commit_message>
<xml_diff>
--- a/output/2026-09-18/enriched_analysis.xlsx
+++ b/output/2026-09-18/enriched_analysis.xlsx
@@ -813,13 +813,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>3.674</v>
+        <v>3.474</v>
       </c>
       <c r="Q2" t="n">
-        <v>2883</v>
+        <v>3049</v>
       </c>
       <c r="R2" t="n">
-        <v>22.6</v>
+        <v>23.9</v>
       </c>
       <c r="S2" t="n">
         <v>75</v>
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.081</v>
+        <v>0.079</v>
       </c>
       <c r="Q3" t="n">
-        <v>2637</v>
+        <v>2696</v>
       </c>
       <c r="R3" t="n">
-        <v>9.06</v>
+        <v>9.25</v>
       </c>
       <c r="S3" t="n">
         <v>36</v>
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.925</v>
+        <v>0.902</v>
       </c>
       <c r="Q4" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="R4" t="n">
-        <v>8.5</v>
+        <v>8.69</v>
       </c>
       <c r="S4" t="n">
         <v>17</v>
@@ -1359,13 +1359,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.552</v>
       </c>
       <c r="Q5" t="n">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="R5" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="S5" t="n">
         <v>22</v>
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.135</v>
+        <v>0.131</v>
       </c>
       <c r="Q6" t="n">
-        <v>2329</v>
+        <v>2393</v>
       </c>
       <c r="R6" t="n">
-        <v>20.4</v>
+        <v>21</v>
       </c>
       <c r="S6" t="n">
         <v>-3</v>
@@ -1723,13 +1723,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.368</v>
+        <v>0.362</v>
       </c>
       <c r="Q7" t="n">
-        <v>2638</v>
+        <v>2683</v>
       </c>
       <c r="R7" t="n">
-        <v>21.6</v>
+        <v>22</v>
       </c>
       <c r="S7" t="n">
         <v>8</v>
@@ -1905,13 +1905,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.059</v>
+        <v>0.055</v>
       </c>
       <c r="Q8" t="n">
-        <v>1392</v>
+        <v>1486</v>
       </c>
       <c r="R8" t="n">
-        <v>18.7</v>
+        <v>20</v>
       </c>
       <c r="S8" t="n">
         <v>55</v>
@@ -2087,10 +2087,10 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.747</v>
+        <v>0.745</v>
       </c>
       <c r="Q9" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
@@ -2267,13 +2267,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>2.908</v>
+        <v>2.866</v>
       </c>
       <c r="Q10" t="n">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="R10" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="S10" t="n">
         <v>5</v>
@@ -2452,10 +2452,10 @@
         <v>0.013</v>
       </c>
       <c r="Q11" t="n">
-        <v>16236</v>
+        <v>16570</v>
       </c>
       <c r="R11" t="n">
-        <v>20.6</v>
+        <v>20.9</v>
       </c>
       <c r="S11" t="n">
         <v>16</v>
@@ -2579,12 +2579,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>DIAMONDYD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>Prataap Snacks Limited</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -2596,181 +2596,181 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F12" t="n">
+        <v>18</v>
+      </c>
+      <c r="G12" t="n">
         <v>13</v>
       </c>
-      <c r="G12" t="n">
-        <v>21</v>
-      </c>
       <c r="H12" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="I12" t="n">
-        <v>631.9</v>
+        <v>1100.4</v>
       </c>
       <c r="J12" t="n">
-        <v>615.76</v>
+        <v>1173.96</v>
       </c>
       <c r="K12" t="n">
-        <v>2.6</v>
+        <v>-6.3</v>
       </c>
       <c r="L12" t="n">
-        <v>64.68000000000001</v>
+        <v>69.75</v>
       </c>
       <c r="M12" t="n">
-        <v>4.67</v>
+        <v>59.58</v>
       </c>
       <c r="N12" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.401</v>
+        <v>2.271</v>
       </c>
       <c r="Q12" t="n">
-        <v>1166</v>
+        <v>2624</v>
       </c>
       <c r="R12" t="n">
-        <v>59.4</v>
+        <v>206</v>
       </c>
       <c r="S12" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="T12" t="n">
-        <v>-0.11</v>
+        <v>19.05</v>
       </c>
       <c r="U12" t="n">
-        <v>23</v>
+        <v>194</v>
       </c>
       <c r="V12" t="n">
-        <v>-0.07000000000000001</v>
+        <v>1.03</v>
       </c>
       <c r="W12" t="n">
-        <v>1.58</v>
+        <v>3.17</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="Y12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z12" t="n">
-        <v>-110</v>
+        <v>3.87</v>
       </c>
       <c r="AA12" t="n">
-        <v>579.95</v>
+        <v>1158.28</v>
       </c>
       <c r="AB12" t="n">
-        <v>514.4</v>
+        <v>1089.6</v>
       </c>
       <c r="AC12" t="n">
-        <v>35</v>
+        <v>16.5</v>
       </c>
       <c r="AD12" t="n">
-        <v>615.760531069126</v>
+        <v>1173.964532439025</v>
       </c>
       <c r="AE12" t="n">
-        <v>2.6</v>
+        <v>-6.3</v>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="AL12" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="AM12" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="AN12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AO12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP12" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="AR12" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="AS12" t="n">
-        <v>2733734</v>
+        <v>0</v>
       </c>
       <c r="AT12" t="n">
-        <v>5220553</v>
+        <v>0</v>
       </c>
       <c r="AU12" t="n">
-        <v>20318705</v>
+        <v>0</v>
       </c>
       <c r="AV12" t="n">
-        <v>24502154</v>
+        <v>586966134</v>
       </c>
       <c r="AW12" t="n">
-        <v>32787234</v>
+        <v>595794044</v>
       </c>
       <c r="AX12" t="n">
-        <v>2733734</v>
+        <v>0</v>
       </c>
       <c r="AY12" t="n">
-        <v>20318705</v>
+        <v>0</v>
       </c>
       <c r="AZ12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BA12" t="n">
         <v>0</v>
       </c>
       <c r="BB12" t="n">
-        <v>0.1345</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DIAMONDYD</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prataap Snacks Limited</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2778,177 +2778,177 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F13" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G13" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="H13" t="n">
         <v>-2</v>
       </c>
       <c r="I13" t="n">
-        <v>1100.4</v>
+        <v>631.9</v>
       </c>
       <c r="J13" t="n">
-        <v>1173.96</v>
+        <v>615.76</v>
       </c>
       <c r="K13" t="n">
-        <v>-6.3</v>
+        <v>2.6</v>
       </c>
       <c r="L13" t="n">
-        <v>69.75</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>59.58</v>
+        <v>4.67</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>2.263</v>
+        <v>0.388</v>
       </c>
       <c r="Q13" t="n">
-        <v>2633</v>
+        <v>1205</v>
       </c>
       <c r="R13" t="n">
-        <v>207</v>
+        <v>61.4</v>
       </c>
       <c r="S13" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="T13" t="n">
-        <v>19.05</v>
+        <v>-0.11</v>
       </c>
       <c r="U13" t="n">
-        <v>194</v>
+        <v>23</v>
       </c>
       <c r="V13" t="n">
-        <v>1.03</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="W13" t="n">
-        <v>3.17</v>
+        <v>1.58</v>
       </c>
       <c r="X13" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>3.87</v>
+        <v>-110</v>
       </c>
       <c r="AA13" t="n">
-        <v>1158.28</v>
+        <v>579.95</v>
       </c>
       <c r="AB13" t="n">
-        <v>1089.6</v>
+        <v>514.4</v>
       </c>
       <c r="AC13" t="n">
-        <v>16.5</v>
+        <v>35</v>
       </c>
       <c r="AD13" t="n">
-        <v>1173.964532439025</v>
+        <v>615.760531069126</v>
       </c>
       <c r="AE13" t="n">
-        <v>-6.3</v>
+        <v>2.6</v>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="AK13" t="n">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="AL13" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="AM13" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="AN13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AP13" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="AQ13" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="AR13" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="AS13" t="n">
-        <v>0</v>
+        <v>2733734</v>
       </c>
       <c r="AT13" t="n">
-        <v>0</v>
+        <v>5220553</v>
       </c>
       <c r="AU13" t="n">
-        <v>0</v>
+        <v>20318705</v>
       </c>
       <c r="AV13" t="n">
-        <v>586966134</v>
+        <v>24502154</v>
       </c>
       <c r="AW13" t="n">
-        <v>595794044</v>
+        <v>32787234</v>
       </c>
       <c r="AX13" t="n">
-        <v>0</v>
+        <v>2733734</v>
       </c>
       <c r="AY13" t="n">
-        <v>0</v>
+        <v>20318705</v>
       </c>
       <c r="AZ13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA13" t="n">
         <v>0</v>
       </c>
       <c r="BB13" t="n">
-        <v>0</v>
+        <v>0.1345</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2960,91 +2960,91 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F14" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G14" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>517.6</v>
+        <v>4811</v>
       </c>
       <c r="J14" t="n">
-        <v>508.08</v>
+        <v>5198.76</v>
       </c>
       <c r="K14" t="n">
-        <v>1.9</v>
+        <v>-7.5</v>
       </c>
       <c r="L14" t="n">
-        <v>62.09</v>
+        <v>67.16</v>
       </c>
       <c r="M14" t="n">
-        <v>2.54</v>
+        <v>7.21</v>
       </c>
       <c r="N14" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>17-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.286</v>
+        <v>0.047</v>
       </c>
       <c r="Q14" t="n">
-        <v>888</v>
+        <v>15426</v>
       </c>
       <c r="R14" t="n">
-        <v>8.74</v>
+        <v>39.3</v>
       </c>
       <c r="S14" t="n">
-        <v>7</v>
+        <v>83</v>
       </c>
       <c r="T14" t="n">
-        <v>30</v>
+        <v>145</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="V14" t="n">
-        <v>14.66</v>
+        <v>27.38</v>
       </c>
       <c r="W14" t="n">
-        <v>14.4</v>
+        <v>25.5</v>
       </c>
       <c r="X14" t="n">
-        <v>0.01</v>
+        <v>0.64</v>
       </c>
       <c r="Y14" t="b">
         <v>1</v>
       </c>
       <c r="Z14" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="AA14" t="n">
-        <v>494.9</v>
+        <v>5679.67</v>
       </c>
       <c r="AB14" t="n">
-        <v>487.98</v>
+        <v>4401.26</v>
       </c>
       <c r="AC14" t="n">
-        <v>19.3</v>
+        <v>37.3</v>
       </c>
       <c r="AD14" t="n">
-        <v>508.0820900006008</v>
+        <v>5198.755988455989</v>
       </c>
       <c r="AE14" t="n">
-        <v>1.9</v>
+        <v>-7.5</v>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
@@ -3059,78 +3059,78 @@
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>17-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="AL14" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="AM14" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>19879002</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>72054758</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>72054758</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>19879002</v>
+      </c>
+      <c r="AZ14" t="n">
         <v>3</v>
       </c>
-      <c r="AO14" t="n">
-        <v>8</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>15</v>
-      </c>
-      <c r="AQ14" t="n">
-        <v>15</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>15</v>
-      </c>
-      <c r="AS14" t="n">
-        <v>8059675</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>17407688</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>25370063</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>25370063</v>
-      </c>
-      <c r="AW14" t="n">
-        <v>25370063</v>
-      </c>
-      <c r="AX14" t="n">
-        <v>8059675</v>
-      </c>
-      <c r="AY14" t="n">
-        <v>25370063</v>
-      </c>
-      <c r="AZ14" t="n">
-        <v>2</v>
-      </c>
       <c r="BA14" t="n">
         <v>0</v>
       </c>
       <c r="BB14" t="n">
-        <v>0.3177</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>SRHHYPOLTD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3142,91 +3142,91 @@
         </is>
       </c>
       <c r="E15" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G15" t="n">
+        <v>21</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>517.6</v>
+      </c>
+      <c r="J15" t="n">
+        <v>508.08</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L15" t="n">
+        <v>62.09</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N15" t="n">
+        <v>15</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>17-09-2026</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>893</v>
+      </c>
+      <c r="R15" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="S15" t="n">
         <v>7</v>
       </c>
-      <c r="F15" t="n">
-        <v>27</v>
-      </c>
-      <c r="G15" t="n">
-        <v>13</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>4811</v>
-      </c>
-      <c r="J15" t="n">
-        <v>5198.76</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-7.5</v>
-      </c>
-      <c r="L15" t="n">
-        <v>67.16</v>
-      </c>
-      <c r="M15" t="n">
-        <v>7.21</v>
-      </c>
-      <c r="N15" t="n">
-        <v>6</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>31-08-2026</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>14954</v>
-      </c>
-      <c r="R15" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="S15" t="n">
-        <v>83</v>
-      </c>
       <c r="T15" t="n">
-        <v>145</v>
+        <v>30</v>
       </c>
       <c r="U15" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>27.38</v>
+        <v>14.66</v>
       </c>
       <c r="W15" t="n">
-        <v>25.5</v>
+        <v>14.4</v>
       </c>
       <c r="X15" t="n">
-        <v>0.64</v>
+        <v>0.01</v>
       </c>
       <c r="Y15" t="b">
         <v>1</v>
       </c>
       <c r="Z15" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="AA15" t="n">
-        <v>5679.67</v>
+        <v>494.9</v>
       </c>
       <c r="AB15" t="n">
-        <v>4401.26</v>
+        <v>487.98</v>
       </c>
       <c r="AC15" t="n">
-        <v>37.3</v>
+        <v>19.3</v>
       </c>
       <c r="AD15" t="n">
-        <v>5198.755988455989</v>
+        <v>508.0820900006008</v>
       </c>
       <c r="AE15" t="n">
-        <v>-7.5</v>
+        <v>1.9</v>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
@@ -3241,67 +3241,67 @@
       </c>
       <c r="AI15" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="AL15" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="AM15" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="AN15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO15" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AP15" t="n">
+        <v>15</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>15</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>15</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>8059675</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>17407688</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>25370063</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>25370063</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>25370063</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>8059675</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>25370063</v>
+      </c>
+      <c r="AZ15" t="n">
         <v>2</v>
       </c>
-      <c r="AQ15" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>19879002</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>72054758</v>
-      </c>
-      <c r="AW15" t="n">
-        <v>72054758</v>
-      </c>
-      <c r="AX15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY15" t="n">
-        <v>19879002</v>
-      </c>
-      <c r="AZ15" t="n">
-        <v>3</v>
-      </c>
       <c r="BA15" t="n">
         <v>0</v>
       </c>
       <c r="BB15" t="n">
-        <v>0</v>
+        <v>0.3177</v>
       </c>
     </row>
     <row r="16">
@@ -3316,7 +3316,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
         <v>25</v>
       </c>
       <c r="H16" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>274</v>
@@ -3359,13 +3359,13 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.151</v>
+        <v>0.155</v>
       </c>
       <c r="Q16" t="n">
-        <v>737</v>
+        <v>717</v>
       </c>
       <c r="R16" t="n">
-        <v>61.6</v>
+        <v>59.9</v>
       </c>
       <c r="S16" t="n">
         <v>3</v>
@@ -3489,16 +3489,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -3506,89 +3506,91 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G17" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H17" t="n">
         <v>-1</v>
       </c>
       <c r="I17" t="n">
-        <v>55.82</v>
+        <v>196.18</v>
       </c>
       <c r="J17" t="n">
-        <v>53.45</v>
+        <v>170.45</v>
       </c>
       <c r="K17" t="n">
-        <v>4.4</v>
+        <v>15.1</v>
       </c>
       <c r="L17" t="n">
-        <v>67.23</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>1.95</v>
+        <v>0.26</v>
       </c>
       <c r="N17" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>1.653</v>
+        <v>0.104</v>
       </c>
       <c r="Q17" t="n">
-        <v>118</v>
-      </c>
-      <c r="R17" t="inlineStr"/>
+        <v>251</v>
+      </c>
+      <c r="R17" t="n">
+        <v>26.9</v>
+      </c>
       <c r="S17" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="T17" t="n">
-        <v>2.47</v>
+        <v>1.87</v>
       </c>
       <c r="U17" t="n">
-        <v>-3779</v>
+        <v>-31</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.05</v>
+        <v>3.36</v>
       </c>
       <c r="W17" t="n">
-        <v>-1.26</v>
+        <v>4.96</v>
       </c>
       <c r="X17" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="Y17" t="b">
         <v>1</v>
       </c>
       <c r="Z17" t="n">
-        <v>3</v>
+        <v>2.97</v>
       </c>
       <c r="AA17" t="n">
-        <v>54.18</v>
+        <v>179.83</v>
       </c>
       <c r="AB17" t="n">
-        <v>55.15</v>
+        <v>162.84</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.6</v>
+        <v>42.8</v>
       </c>
       <c r="AD17" t="n">
-        <v>53.44741172107844</v>
+        <v>170.4518641810919</v>
       </c>
       <c r="AE17" t="n">
-        <v>4.4</v>
+        <v>15.1</v>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
@@ -3598,87 +3600,87 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>05-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="AL17" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="AM17" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="AN17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AP17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AQ17" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="AR17" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="AS17" t="n">
-        <v>789002</v>
+        <v>0</v>
       </c>
       <c r="AT17" t="n">
-        <v>1412746</v>
+        <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>5992468</v>
+        <v>5120374</v>
       </c>
       <c r="AV17" t="n">
-        <v>19457263</v>
+        <v>5120374</v>
       </c>
       <c r="AW17" t="n">
-        <v>19457263</v>
+        <v>5120374</v>
       </c>
       <c r="AX17" t="n">
-        <v>789002</v>
+        <v>0</v>
       </c>
       <c r="AY17" t="n">
-        <v>5992468</v>
+        <v>5120374</v>
       </c>
       <c r="AZ17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA17" t="n">
         <v>0</v>
       </c>
       <c r="BB17" t="n">
-        <v>0.1317</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>OBCL LIMITED</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -3686,87 +3688,85 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F18" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H18" t="n">
         <v>-1</v>
       </c>
       <c r="I18" t="n">
-        <v>210.04</v>
+        <v>55.82</v>
       </c>
       <c r="J18" t="n">
-        <v>210</v>
+        <v>53.45</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>4.4</v>
       </c>
       <c r="L18" t="n">
-        <v>67.04000000000001</v>
+        <v>67.23</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.95</v>
       </c>
       <c r="N18" t="n">
         <v>11</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>15-09-2026</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.284</v>
+        <v>1.625</v>
       </c>
       <c r="Q18" t="n">
-        <v>197</v>
-      </c>
-      <c r="R18" t="n">
-        <v>24.4</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="T18" t="n">
-        <v>0.03</v>
+        <v>2.47</v>
       </c>
       <c r="U18" t="n">
-        <v>16</v>
+        <v>-3779</v>
       </c>
       <c r="V18" t="n">
-        <v>0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="W18" t="n">
-        <v>7.91</v>
+        <v>-1.26</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="Y18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z18" t="n">
-        <v>3.16</v>
+        <v>3</v>
       </c>
       <c r="AA18" t="n">
-        <v>209.31</v>
+        <v>54.18</v>
       </c>
       <c r="AB18" t="n">
-        <v>195.66</v>
+        <v>55.15</v>
       </c>
       <c r="AC18" t="n">
-        <v>8.5</v>
+        <v>0.6</v>
       </c>
       <c r="AD18" t="n">
-        <v>210.0038192234246</v>
+        <v>53.44741172107844</v>
       </c>
       <c r="AE18" t="n">
-        <v>0</v>
+        <v>4.4</v>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
@@ -3785,31 +3785,31 @@
       </c>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>15-09-2026</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="AL18" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="AM18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AP18" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AQ18" t="n">
         <v>11</v>
@@ -3818,25 +3818,25 @@
         <v>11</v>
       </c>
       <c r="AS18" t="n">
-        <v>1373791</v>
+        <v>789002</v>
       </c>
       <c r="AT18" t="n">
-        <v>2710295</v>
+        <v>1412746</v>
       </c>
       <c r="AU18" t="n">
-        <v>3426986</v>
+        <v>5992468</v>
       </c>
       <c r="AV18" t="n">
-        <v>5608572</v>
+        <v>19457263</v>
       </c>
       <c r="AW18" t="n">
-        <v>5608572</v>
+        <v>19457263</v>
       </c>
       <c r="AX18" t="n">
-        <v>1373791</v>
+        <v>789002</v>
       </c>
       <c r="AY18" t="n">
-        <v>3426986</v>
+        <v>5992468</v>
       </c>
       <c r="AZ18" t="n">
         <v>1</v>
@@ -3845,7 +3845,7 @@
         <v>0</v>
       </c>
       <c r="BB18" t="n">
-        <v>0.4009</v>
+        <v>0.1317</v>
       </c>
     </row>
     <row r="19">
@@ -3906,7 +3906,7 @@
         <v>0.33</v>
       </c>
       <c r="Q19" t="n">
-        <v>3870</v>
+        <v>3868</v>
       </c>
       <c r="R19" t="n">
         <v>87.09999999999999</v>
@@ -4033,12 +4033,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -4050,96 +4050,96 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G20" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H20" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>196.18</v>
+        <v>365.15</v>
       </c>
       <c r="J20" t="n">
-        <v>170.45</v>
+        <v>338.1</v>
       </c>
       <c r="K20" t="n">
-        <v>15.1</v>
+        <v>8</v>
       </c>
       <c r="L20" t="n">
-        <v>67.54000000000001</v>
+        <v>66.73</v>
       </c>
       <c r="M20" t="n">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="N20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.098</v>
+        <v>0.079</v>
       </c>
       <c r="Q20" t="n">
-        <v>264</v>
+        <v>430</v>
       </c>
       <c r="R20" t="n">
-        <v>28.2</v>
+        <v>12.7</v>
       </c>
       <c r="S20" t="n">
+        <v>-8</v>
+      </c>
+      <c r="T20" t="n">
         <v>24</v>
       </c>
-      <c r="T20" t="n">
-        <v>1.87</v>
-      </c>
       <c r="U20" t="n">
-        <v>-31</v>
+        <v>33</v>
       </c>
       <c r="V20" t="n">
-        <v>3.36</v>
+        <v>14.36</v>
       </c>
       <c r="W20" t="n">
-        <v>4.96</v>
+        <v>9.94</v>
       </c>
       <c r="X20" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="Y20" t="b">
         <v>1</v>
       </c>
       <c r="Z20" t="n">
-        <v>2.97</v>
+        <v>18</v>
       </c>
       <c r="AA20" t="n">
-        <v>179.83</v>
+        <v>346.89</v>
       </c>
       <c r="AB20" t="n">
-        <v>162.84</v>
+        <v>266.32</v>
       </c>
       <c r="AC20" t="n">
-        <v>42.8</v>
+        <v>99.8</v>
       </c>
       <c r="AD20" t="n">
-        <v>170.4518641810919</v>
+        <v>338.1</v>
       </c>
       <c r="AE20" t="n">
-        <v>15.1</v>
+        <v>8</v>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AH20" t="inlineStr">
@@ -4149,22 +4149,22 @@
       </c>
       <c r="AI20" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AK20" t="n">
         <v>0</v>
       </c>
       <c r="AL20" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="AM20" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4173,13 +4173,13 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AQ20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AR20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AS20" t="n">
         <v>0</v>
@@ -4188,22 +4188,22 @@
         <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>5120374</v>
+        <v>0</v>
       </c>
       <c r="AV20" t="n">
-        <v>5120374</v>
+        <v>3381000</v>
       </c>
       <c r="AW20" t="n">
-        <v>5120374</v>
+        <v>3381000</v>
       </c>
       <c r="AX20" t="n">
         <v>0</v>
       </c>
       <c r="AY20" t="n">
-        <v>5120374</v>
+        <v>0</v>
       </c>
       <c r="AZ20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BA20" t="n">
         <v>0</v>
@@ -4215,12 +4215,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -4232,157 +4232,157 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F21" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="G21" t="n">
         <v>21</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I21" t="n">
-        <v>365.15</v>
+        <v>210.04</v>
       </c>
       <c r="J21" t="n">
-        <v>338.1</v>
+        <v>210</v>
       </c>
       <c r="K21" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>66.73</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>0.34</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="N21" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.079</v>
+        <v>0.289</v>
       </c>
       <c r="Q21" t="n">
-        <v>430</v>
+        <v>194</v>
       </c>
       <c r="R21" t="n">
-        <v>12.7</v>
+        <v>24.1</v>
       </c>
       <c r="S21" t="n">
-        <v>-8</v>
+        <v>12</v>
       </c>
       <c r="T21" t="n">
-        <v>24</v>
+        <v>0.03</v>
       </c>
       <c r="U21" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="V21" t="n">
-        <v>14.36</v>
+        <v>0.03</v>
       </c>
       <c r="W21" t="n">
-        <v>9.94</v>
+        <v>7.91</v>
       </c>
       <c r="X21" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>18</v>
+        <v>3.16</v>
       </c>
       <c r="AA21" t="n">
-        <v>346.89</v>
+        <v>209.31</v>
       </c>
       <c r="AB21" t="n">
-        <v>266.32</v>
+        <v>195.66</v>
       </c>
       <c r="AC21" t="n">
-        <v>99.8</v>
+        <v>8.5</v>
       </c>
       <c r="AD21" t="n">
-        <v>338.1</v>
+        <v>210.0038192234246</v>
       </c>
       <c r="AE21" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AI21" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="AL21" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="AM21" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="AN21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AP21" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AQ21" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AR21" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AS21" t="n">
-        <v>0</v>
+        <v>1373791</v>
       </c>
       <c r="AT21" t="n">
-        <v>0</v>
+        <v>2710295</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>3426986</v>
       </c>
       <c r="AV21" t="n">
-        <v>3381000</v>
+        <v>5608572</v>
       </c>
       <c r="AW21" t="n">
-        <v>3381000</v>
+        <v>5608572</v>
       </c>
       <c r="AX21" t="n">
-        <v>0</v>
+        <v>1373791</v>
       </c>
       <c r="AY21" t="n">
-        <v>0</v>
+        <v>3426986</v>
       </c>
       <c r="AZ21" t="n">
         <v>1</v>
@@ -4391,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="BB21" t="n">
-        <v>0</v>
+        <v>0.4009</v>
       </c>
     </row>
     <row r="22">
@@ -4449,13 +4449,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>1.064</v>
+        <v>1.074</v>
       </c>
       <c r="Q22" t="n">
-        <v>9650</v>
+        <v>9562</v>
       </c>
       <c r="R22" t="n">
-        <v>12.8</v>
+        <v>12.6</v>
       </c>
       <c r="S22" t="n">
         <v>-12</v>
@@ -4631,13 +4631,13 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.511</v>
+        <v>0.5</v>
       </c>
       <c r="Q23" t="n">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="R23" t="n">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="S23" t="n">
         <v>-1</v>
@@ -4816,10 +4816,10 @@
         <v>0.136</v>
       </c>
       <c r="Q24" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="R24" t="n">
-        <v>5.92</v>
+        <v>5.94</v>
       </c>
       <c r="S24" t="n">
         <v>118</v>
@@ -4994,10 +4994,10 @@
         <v>0.007</v>
       </c>
       <c r="Q25" t="n">
-        <v>5611</v>
+        <v>5682</v>
       </c>
       <c r="R25" t="n">
-        <v>9.48</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="S25" t="n">
         <v>43</v>
@@ -5173,13 +5173,13 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.113</v>
+        <v>0.112</v>
       </c>
       <c r="Q26" t="n">
-        <v>1551</v>
+        <v>1567</v>
       </c>
       <c r="R26" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="S26" t="n">
         <v>581</v>
@@ -5353,13 +5353,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.616</v>
+        <v>0.578</v>
       </c>
       <c r="Q27" t="n">
-        <v>2213</v>
+        <v>2361</v>
       </c>
       <c r="R27" t="n">
-        <v>655</v>
+        <v>698</v>
       </c>
       <c r="S27" t="n">
         <v>3</v>
@@ -5535,13 +5535,13 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.058</v>
+        <v>0.059</v>
       </c>
       <c r="Q28" t="n">
-        <v>1890</v>
+        <v>1870</v>
       </c>
       <c r="R28" t="n">
-        <v>43.4</v>
+        <v>42.9</v>
       </c>
       <c r="S28" t="n">
         <v>20</v>
@@ -5717,13 +5717,13 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0.465</v>
+        <v>0.438</v>
       </c>
       <c r="Q29" t="n">
-        <v>398</v>
+        <v>422</v>
       </c>
       <c r="R29" t="n">
-        <v>36.9</v>
+        <v>39.1</v>
       </c>
       <c r="S29" t="n">
         <v>21</v>
@@ -5902,7 +5902,7 @@
         <v>0.044</v>
       </c>
       <c r="Q30" t="n">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="R30" t="n">
         <v>101</v>
@@ -6081,13 +6081,13 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="Q31" t="n">
-        <v>3504</v>
+        <v>3460</v>
       </c>
       <c r="R31" t="n">
-        <v>20.8</v>
+        <v>20.5</v>
       </c>
       <c r="S31" t="n">
         <v>-4</v>
@@ -6266,10 +6266,10 @@
         <v>0.064</v>
       </c>
       <c r="Q32" t="n">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="R32" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="S32" t="n">
         <v>19</v>
@@ -6448,10 +6448,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="Q33" t="n">
-        <v>52307</v>
+        <v>53146</v>
       </c>
       <c r="R33" t="n">
-        <v>44.3</v>
+        <v>45</v>
       </c>
       <c r="S33" t="n">
         <v>5</v>
@@ -6630,10 +6630,10 @@
         <v>0.042</v>
       </c>
       <c r="Q34" t="n">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="R34" t="n">
-        <v>48.1</v>
+        <v>47.9</v>
       </c>
       <c r="S34" t="n">
         <v>7</v>
@@ -6809,13 +6809,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.673</v>
+        <v>0.661</v>
       </c>
       <c r="Q35" t="n">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="R35" t="n">
-        <v>1094</v>
+        <v>1111</v>
       </c>
       <c r="S35" t="n">
         <v>-61</v>
@@ -6990,10 +6990,10 @@
         <v>0.052</v>
       </c>
       <c r="Q36" t="n">
-        <v>5074</v>
+        <v>5106</v>
       </c>
       <c r="R36" t="n">
-        <v>33.1</v>
+        <v>33.3</v>
       </c>
       <c r="S36" t="n">
         <v>-25</v>
@@ -7172,7 +7172,7 @@
         <v>0.027</v>
       </c>
       <c r="Q37" t="n">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="n">
@@ -7349,13 +7349,13 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.995</v>
+        <v>0.961</v>
       </c>
       <c r="Q38" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="R38" t="n">
-        <v>5.82</v>
+        <v>6.01</v>
       </c>
       <c r="S38" t="n">
         <v>31</v>
@@ -7527,13 +7527,13 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.532</v>
+        <v>0.527</v>
       </c>
       <c r="Q39" t="n">
-        <v>3635</v>
+        <v>3669</v>
       </c>
       <c r="R39" t="n">
-        <v>25.4</v>
+        <v>25.7</v>
       </c>
       <c r="S39" t="n">
         <v>2</v>
@@ -7712,10 +7712,10 @@
         <v>0.035</v>
       </c>
       <c r="Q40" t="n">
-        <v>3157</v>
+        <v>3147</v>
       </c>
       <c r="R40" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="S40" t="n">
         <v>17</v>
@@ -7891,13 +7891,13 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.206</v>
+        <v>0.211</v>
       </c>
       <c r="Q41" t="n">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="R41" t="n">
-        <v>25.9</v>
+        <v>25.4</v>
       </c>
       <c r="S41" t="n">
         <v>21</v>
@@ -8073,13 +8073,13 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>2.256</v>
+        <v>2.246</v>
       </c>
       <c r="Q42" t="n">
-        <v>24712</v>
+        <v>24816</v>
       </c>
       <c r="R42" t="n">
-        <v>31.2</v>
+        <v>31.4</v>
       </c>
       <c r="S42" t="n">
         <v>-2</v>
@@ -8203,16 +8203,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DOLLAR</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DOLLAR INDUSTRIES LIMITED</t>
+          <t>BMW VENTURES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -8220,121 +8220,121 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G43" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I43" t="n">
-        <v>267</v>
+        <v>50.22</v>
       </c>
       <c r="J43" t="n">
-        <v>269.7</v>
+        <v>56.66</v>
       </c>
       <c r="K43" t="n">
-        <v>-1</v>
+        <v>-11.4</v>
       </c>
       <c r="L43" t="n">
-        <v>73.09</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="M43" t="n">
-        <v>1.48</v>
+        <v>1.9</v>
       </c>
       <c r="N43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>16-08-2026</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.098</v>
+        <v>0.433</v>
       </c>
       <c r="Q43" t="n">
-        <v>1514</v>
+        <v>439</v>
       </c>
       <c r="R43" t="n">
-        <v>13.7</v>
+        <v>11</v>
       </c>
       <c r="S43" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="T43" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="U43" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V43" t="n">
-        <v>4.31</v>
+        <v>1.22</v>
       </c>
       <c r="W43" t="n">
-        <v>13.6</v>
+        <v>12</v>
       </c>
       <c r="X43" t="n">
-        <v>0.28</v>
+        <v>0.58</v>
       </c>
       <c r="Y43" t="b">
         <v>1</v>
       </c>
       <c r="Z43" t="n">
-        <v>12</v>
+        <v>3.4</v>
       </c>
       <c r="AA43" t="n">
-        <v>267.63</v>
+        <v>56.88</v>
       </c>
       <c r="AB43" t="n">
-        <v>288.6</v>
+        <v>58.37</v>
       </c>
       <c r="AC43" t="n">
-        <v>8.300000000000001</v>
+        <v>-17.5</v>
       </c>
       <c r="AD43" t="n">
-        <v>269.7</v>
+        <v>57.35626428571429</v>
       </c>
       <c r="AE43" t="n">
-        <v>-1</v>
+        <v>-12.4</v>
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AG43" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AH43" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AI43" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="AJ43" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>16-08-2026</t>
         </is>
       </c>
       <c r="AK43" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AL43" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="AM43" t="n">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="AN43" t="n">
         <v>0</v>
@@ -8346,10 +8346,10 @@
         <v>0</v>
       </c>
       <c r="AQ43" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AS43" t="n">
         <v>0</v>
@@ -8361,10 +8361,10 @@
         <v>0</v>
       </c>
       <c r="AV43" t="n">
-        <v>0</v>
+        <v>24089631</v>
       </c>
       <c r="AW43" t="n">
-        <v>14833500</v>
+        <v>24089631</v>
       </c>
       <c r="AX43" t="n">
         <v>0</v>
@@ -8385,16 +8385,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>DOLLAR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>VIVIANA POWER TECH LIMITED</t>
+          <t>DOLLAR INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -8402,85 +8402,87 @@
         </is>
       </c>
       <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>18</v>
+      </c>
+      <c r="G44" t="n">
         <v>5</v>
       </c>
-      <c r="F44" t="n">
-        <v>19</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
       <c r="H44" t="n">
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>724.7</v>
+        <v>267</v>
       </c>
       <c r="J44" t="n">
-        <v>815.16</v>
+        <v>269.7</v>
       </c>
       <c r="K44" t="n">
-        <v>-11.1</v>
+        <v>-1</v>
       </c>
       <c r="L44" t="n">
-        <v>73.2</v>
+        <v>73.09</v>
       </c>
       <c r="M44" t="n">
-        <v>1.24</v>
+        <v>1.48</v>
       </c>
       <c r="N44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.169</v>
+        <v>0.096</v>
       </c>
       <c r="Q44" t="n">
-        <v>734</v>
+        <v>1536</v>
       </c>
       <c r="R44" t="n">
-        <v>13.3</v>
+        <v>13.9</v>
       </c>
       <c r="S44" t="n">
-        <v>185</v>
+        <v>6</v>
       </c>
       <c r="T44" t="n">
-        <v>11.55</v>
+        <v>46</v>
       </c>
       <c r="U44" t="n">
-        <v>204</v>
+        <v>18</v>
       </c>
       <c r="V44" t="n">
-        <v>6.84</v>
+        <v>4.31</v>
       </c>
       <c r="W44" t="n">
-        <v>50.7</v>
+        <v>13.6</v>
       </c>
       <c r="X44" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.28</v>
       </c>
       <c r="Y44" t="b">
         <v>1</v>
       </c>
       <c r="Z44" t="n">
-        <v>16.07</v>
+        <v>12</v>
       </c>
       <c r="AA44" t="n">
-        <v>730.95</v>
-      </c>
-      <c r="AB44" t="inlineStr"/>
+        <v>267.63</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>288.6</v>
+      </c>
       <c r="AC44" t="n">
-        <v>-20.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AD44" t="n">
-        <v>815.1570095913809</v>
+        <v>269.7</v>
       </c>
       <c r="AE44" t="n">
-        <v>-11.1</v>
+        <v>-1</v>
       </c>
       <c r="AF44" t="inlineStr">
         <is>
@@ -8499,22 +8501,22 @@
       </c>
       <c r="AI44" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AJ44" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AK44" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AL44" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AM44" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="AN44" t="n">
         <v>0</v>
@@ -8544,7 +8546,7 @@
         <v>0</v>
       </c>
       <c r="AW44" t="n">
-        <v>3623803</v>
+        <v>14833500</v>
       </c>
       <c r="AX44" t="n">
         <v>0</v>
@@ -8553,7 +8555,7 @@
         <v>0</v>
       </c>
       <c r="AZ44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BA44" t="n">
         <v>0</v>
@@ -8565,16 +8567,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BMW VENTURES LIMITED</t>
+          <t>VIVIANA POWER TECH LIMITED</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -8591,151 +8593,149 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>50.22</v>
+        <v>724.7</v>
       </c>
       <c r="J45" t="n">
-        <v>60.15</v>
+        <v>815.16</v>
       </c>
       <c r="K45" t="n">
-        <v>-16.5</v>
+        <v>-11.1</v>
       </c>
       <c r="L45" t="n">
-        <v>73.01000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="M45" t="n">
-        <v>0.9</v>
+        <v>1.24</v>
       </c>
       <c r="N45" t="n">
+        <v>3</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>729</v>
+      </c>
+      <c r="R45" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="S45" t="n">
+        <v>185</v>
+      </c>
+      <c r="T45" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="U45" t="n">
+        <v>204</v>
+      </c>
+      <c r="V45" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="W45" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="X45" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="Y45" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>16.07</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>730.95</v>
+      </c>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="n">
+        <v>-20.3</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>815.1570095913809</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>-11.1</v>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>Stale Accumulation</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr">
+        <is>
+          <t>Late — Poor Entry</t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>19-06-2026</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="AK45" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>91</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>81</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>3623803</v>
+      </c>
+      <c r="AX45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ45" t="n">
         <v>2</v>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>06-08-2026</t>
-        </is>
-      </c>
-      <c r="P45" t="n">
-        <v>0.207</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>435</v>
-      </c>
-      <c r="R45" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="S45" t="n">
-        <v>19</v>
-      </c>
-      <c r="T45" t="n">
-        <v>21</v>
-      </c>
-      <c r="U45" t="n">
-        <v>20</v>
-      </c>
-      <c r="V45" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="W45" t="n">
-        <v>12</v>
-      </c>
-      <c r="X45" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="Y45" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="AA45" t="n">
-        <v>56.88</v>
-      </c>
-      <c r="AB45" t="n">
-        <v>58.37</v>
-      </c>
-      <c r="AC45" t="n">
-        <v>-17.5</v>
-      </c>
-      <c r="AD45" t="n">
-        <v>60.1322085106383</v>
-      </c>
-      <c r="AE45" t="n">
-        <v>-16.5</v>
-      </c>
-      <c r="AF45" t="inlineStr">
-        <is>
-          <t>Aging</t>
-        </is>
-      </c>
-      <c r="AG45" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AH45" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AI45" t="inlineStr">
-        <is>
-          <t>05-08-2026</t>
-        </is>
-      </c>
-      <c r="AJ45" t="inlineStr">
-        <is>
-          <t>06-08-2026</t>
-        </is>
-      </c>
-      <c r="AK45" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL45" t="n">
-        <v>44</v>
-      </c>
-      <c r="AM45" t="n">
-        <v>43</v>
-      </c>
-      <c r="AN45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ45" t="n">
-        <v>3</v>
-      </c>
-      <c r="AR45" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV45" t="n">
-        <v>14131069</v>
-      </c>
-      <c r="AW45" t="n">
-        <v>14131069</v>
-      </c>
-      <c r="AX45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY45" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ45" t="n">
-        <v>1</v>
       </c>
       <c r="BA45" t="n">
         <v>0</v>
@@ -8802,10 +8802,10 @@
         <v>0.043</v>
       </c>
       <c r="Q46" t="n">
-        <v>1591</v>
+        <v>1599</v>
       </c>
       <c r="R46" t="n">
-        <v>20.8</v>
+        <v>20.9</v>
       </c>
       <c r="S46" t="n">
         <v>10</v>
@@ -8981,13 +8981,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.185</v>
+        <v>0.177</v>
       </c>
       <c r="Q47" t="n">
-        <v>1733</v>
+        <v>1809</v>
       </c>
       <c r="R47" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="S47" t="n">
         <v>-3</v>
@@ -9163,13 +9163,13 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.13</v>
+        <v>0.128</v>
       </c>
       <c r="Q48" t="n">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="R48" t="n">
-        <v>13.5</v>
+        <v>13.8</v>
       </c>
       <c r="S48" t="n">
         <v>61</v>
@@ -9346,10 +9346,10 @@
         <v>0.039</v>
       </c>
       <c r="Q49" t="n">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="R49" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="n">
@@ -9517,13 +9517,13 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.248</v>
+        <v>0.246</v>
       </c>
       <c r="Q50" t="n">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="R50" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="S50" t="n">
         <v>16</v>
@@ -9699,13 +9699,13 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="Q51" t="n">
-        <v>8873</v>
+        <v>8988</v>
       </c>
       <c r="R51" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="S51" t="n">
         <v>21</v>
@@ -9881,13 +9881,13 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>0.377</v>
+        <v>0.376</v>
       </c>
       <c r="Q52" t="n">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="R52" t="n">
-        <v>97.40000000000001</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="S52" t="n">
         <v>246</v>
@@ -10066,10 +10066,10 @@
         <v>0.008</v>
       </c>
       <c r="Q53" t="n">
-        <v>115107</v>
+        <v>114944</v>
       </c>
       <c r="R53" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="S53" t="n">
         <v>18</v>
@@ -10245,13 +10245,13 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>0.139</v>
+        <v>0.136</v>
       </c>
       <c r="Q54" t="n">
-        <v>1660</v>
+        <v>1694</v>
       </c>
       <c r="R54" t="n">
-        <v>30</v>
+        <v>30.6</v>
       </c>
       <c r="S54" t="n">
         <v>39</v>
@@ -10427,13 +10427,13 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>0.028</v>
+        <v>0.027</v>
       </c>
       <c r="Q55" t="n">
-        <v>971</v>
+        <v>1000</v>
       </c>
       <c r="R55" t="n">
-        <v>26.4</v>
+        <v>27.2</v>
       </c>
       <c r="S55" t="n">
         <v>9</v>
@@ -10979,140 +10979,140 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>DIAMONDYD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>Prataap Snacks Limited</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>631.9</v>
+        <v>1100.4</v>
       </c>
       <c r="D12" t="n">
-        <v>615.76</v>
+        <v>1173.96</v>
       </c>
       <c r="E12" t="n">
-        <v>2.6</v>
+        <v>-6.3</v>
       </c>
       <c r="F12" t="n">
-        <v>64.68000000000001</v>
+        <v>69.75</v>
       </c>
       <c r="G12" t="n">
-        <v>4.67</v>
+        <v>59.58</v>
       </c>
       <c r="H12" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DIAMONDYD</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prataap Snacks Limited</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1100.4</v>
+        <v>631.9</v>
       </c>
       <c r="D13" t="n">
-        <v>1173.96</v>
+        <v>615.76</v>
       </c>
       <c r="E13" t="n">
-        <v>-6.3</v>
+        <v>2.6</v>
       </c>
       <c r="F13" t="n">
-        <v>69.75</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>59.58</v>
+        <v>4.67</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>517.6</v>
+        <v>4811</v>
       </c>
       <c r="D14" t="n">
-        <v>508.08</v>
+        <v>5198.76</v>
       </c>
       <c r="E14" t="n">
-        <v>1.9</v>
+        <v>-7.5</v>
       </c>
       <c r="F14" t="n">
-        <v>62.09</v>
+        <v>67.16</v>
       </c>
       <c r="G14" t="n">
-        <v>2.54</v>
+        <v>7.21</v>
       </c>
       <c r="H14" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>17-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>SRHHYPOLTD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4811</v>
+        <v>517.6</v>
       </c>
       <c r="D15" t="n">
-        <v>5198.76</v>
+        <v>508.08</v>
       </c>
       <c r="E15" t="n">
-        <v>-7.5</v>
+        <v>1.9</v>
       </c>
       <c r="F15" t="n">
-        <v>67.16</v>
+        <v>62.09</v>
       </c>
       <c r="G15" t="n">
-        <v>7.21</v>
+        <v>2.54</v>
       </c>
       <c r="H15" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
     </row>
@@ -11154,70 +11154,70 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>55.82</v>
+        <v>196.18</v>
       </c>
       <c r="D17" t="n">
-        <v>53.45</v>
+        <v>170.45</v>
       </c>
       <c r="E17" t="n">
-        <v>4.4</v>
+        <v>15.1</v>
       </c>
       <c r="F17" t="n">
-        <v>67.23</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>1.95</v>
+        <v>0.26</v>
       </c>
       <c r="H17" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>OBCL LIMITED</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>210.04</v>
+        <v>55.82</v>
       </c>
       <c r="D18" t="n">
-        <v>210</v>
+        <v>53.45</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>4.4</v>
       </c>
       <c r="F18" t="n">
-        <v>67.04000000000001</v>
+        <v>67.23</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.95</v>
       </c>
       <c r="H18" t="n">
         <v>11</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>15-09-2026</t>
         </is>
       </c>
     </row>
@@ -11259,70 +11259,70 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>196.18</v>
+        <v>365.15</v>
       </c>
       <c r="D20" t="n">
-        <v>170.45</v>
+        <v>338.1</v>
       </c>
       <c r="E20" t="n">
-        <v>15.1</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>67.54000000000001</v>
+        <v>66.73</v>
       </c>
       <c r="G20" t="n">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>365.15</v>
+        <v>210.04</v>
       </c>
       <c r="D21" t="n">
-        <v>338.1</v>
+        <v>210</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>66.73</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>0.34</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
     </row>
@@ -12064,105 +12064,105 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DOLLAR</t>
+          <t>BMWVENTLTD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DOLLAR INDUSTRIES LIMITED</t>
+          <t>BMW VENTURES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>267</v>
+        <v>50.22</v>
       </c>
       <c r="D43" t="n">
-        <v>269.7</v>
+        <v>56.66</v>
       </c>
       <c r="E43" t="n">
-        <v>-1</v>
+        <v>-11.4</v>
       </c>
       <c r="F43" t="n">
-        <v>73.09</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="G43" t="n">
-        <v>1.48</v>
+        <v>1.9</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>16-08-2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>DOLLAR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>VIVIANA POWER TECH LIMITED</t>
+          <t>DOLLAR INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>724.7</v>
+        <v>267</v>
       </c>
       <c r="D44" t="n">
-        <v>815.16</v>
+        <v>269.7</v>
       </c>
       <c r="E44" t="n">
-        <v>-11.1</v>
+        <v>-1</v>
       </c>
       <c r="F44" t="n">
-        <v>73.2</v>
+        <v>73.09</v>
       </c>
       <c r="G44" t="n">
-        <v>1.24</v>
+        <v>1.48</v>
       </c>
       <c r="H44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BMWVENTLTD</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BMW VENTURES LIMITED</t>
+          <t>VIVIANA POWER TECH LIMITED</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>50.22</v>
+        <v>724.7</v>
       </c>
       <c r="D45" t="n">
-        <v>60.15</v>
+        <v>815.16</v>
       </c>
       <c r="E45" t="n">
-        <v>-16.5</v>
+        <v>-11.1</v>
       </c>
       <c r="F45" t="n">
-        <v>73.01000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="G45" t="n">
-        <v>0.9</v>
+        <v>1.24</v>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>06-08-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
     </row>

</xml_diff>